<commit_message>
them 2 cot ma khach hang vao bang property
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_matrix_dot1.xlsx
+++ b/docs/SLMS2026_import_matrix_dot1.xlsx
@@ -402,9 +402,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A9"/>
-  <cols>
-    <col min="1" max="1" width="41.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -461,18 +458,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J60"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2161,10 +2146,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B20"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2332,24 +2313,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O51"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="17.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="17.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="17.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:Q51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2397,6 +2361,12 @@
       <c r="O1" t="str">
         <v>Mô tả chi tiết</v>
       </c>
+      <c r="P1" t="str">
+        <v>Mã khách hàng điện</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Mã khách hàng nước</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2444,6 +2414,12 @@
       <c r="O2" t="str">
         <v>MTX#01 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2491,6 +2467,12 @@
       <c r="O3" t="str">
         <v>MTX#02 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2538,6 +2520,12 @@
       <c r="O4" t="str">
         <v>MTX#03 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2585,6 +2573,12 @@
       <c r="O5" t="str">
         <v>MTX#04 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2632,6 +2626,12 @@
       <c r="O6" t="str">
         <v>MTX#05 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2679,6 +2679,12 @@
       <c r="O7" t="str">
         <v>MTX#06 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2726,6 +2732,12 @@
       <c r="O8" t="str">
         <v>MTX#07 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2773,6 +2785,12 @@
       <c r="O9" t="str">
         <v>MTX#08 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2820,6 +2838,12 @@
       <c r="O10" t="str">
         <v>MTX#09 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2867,6 +2891,12 @@
       <c r="O11" t="str">
         <v>MTX#10 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2914,6 +2944,12 @@
       <c r="O12" t="str">
         <v>MTX#11 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2961,6 +2997,12 @@
       <c r="O13" t="str">
         <v>MTX#12 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -3008,6 +3050,12 @@
       <c r="O14" t="str">
         <v>MTX#13 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -3055,6 +3103,12 @@
       <c r="O15" t="str">
         <v>MTX#14 NGUYEN_CAN full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -3102,6 +3156,12 @@
       <c r="O16" t="str">
         <v>MTX#15 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -3149,6 +3209,12 @@
       <c r="O17" t="str">
         <v>MTX#16 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -3196,6 +3262,12 @@
       <c r="O18" t="str">
         <v>MTX#17 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -3243,6 +3315,12 @@
       <c r="O19" t="str">
         <v>MTX#18 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -3290,6 +3368,12 @@
       <c r="O20" t="str">
         <v>MTX#19 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -3337,6 +3421,12 @@
       <c r="O21" t="str">
         <v>MTX#20 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3384,6 +3474,12 @@
       <c r="O22" t="str">
         <v>MTX#21 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -3431,6 +3527,12 @@
       <c r="O23" t="str">
         <v>MTX#22 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -3478,6 +3580,12 @@
       <c r="O24" t="str">
         <v>MTX#23 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -3525,6 +3633,12 @@
       <c r="O25" t="str">
         <v>MTX#24 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -3572,6 +3686,12 @@
       <c r="O26" t="str">
         <v>MTX#25 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -3619,6 +3739,12 @@
       <c r="O27" t="str">
         <v>MTX#26 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3666,6 +3792,12 @@
       <c r="O28" t="str">
         <v>MTX#27 NGUYEN_CAN NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3713,6 +3845,12 @@
       <c r="O29" t="str">
         <v>MTX#28 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -3760,6 +3898,12 @@
       <c r="O30" t="str">
         <v>MTX#29 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -3807,6 +3951,12 @@
       <c r="O31" t="str">
         <v>MTX#30 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -3854,6 +4004,12 @@
       <c r="O32" t="str">
         <v>MTX#31 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3901,6 +4057,12 @@
       <c r="O33" t="str">
         <v>MTX#32 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -3948,6 +4110,12 @@
       <c r="O34" t="str">
         <v>MTX#33 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3995,6 +4163,12 @@
       <c r="O35" t="str">
         <v>MTX#34 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4042,6 +4216,12 @@
       <c r="O36" t="str">
         <v>MTX#35 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4089,6 +4269,12 @@
       <c r="O37" t="str">
         <v>MTX#36 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -4136,6 +4322,12 @@
       <c r="O38" t="str">
         <v>MTX#37 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -4183,6 +4375,12 @@
       <c r="O39" t="str">
         <v>MTX#38 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -4230,6 +4428,12 @@
       <c r="O40" t="str">
         <v>MTX#39 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -4277,6 +4481,12 @@
       <c r="O41" t="str">
         <v>MTX#40 NGUYEN_CAN không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -4324,6 +4534,12 @@
       <c r="O42" t="str">
         <v>MTX#41 THEO_PHONG full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -4371,6 +4587,12 @@
       <c r="O43" t="str">
         <v>MTX#42 THEO_PHONG full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -4418,6 +4640,12 @@
       <c r="O44" t="str">
         <v>MTX#43 THEO_PHONG full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -4465,6 +4693,12 @@
       <c r="O45" t="str">
         <v>MTX#44 THEO_PHONG full NT — RENO. NT khai thác = TB mua mới đợt 2 (FULL). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -4512,6 +4746,12 @@
       <c r="O46" t="str">
         <v>MTX#45 THEO_PHONG NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P46" t="str">
+        <v/>
+      </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -4559,6 +4799,12 @@
       <c r="O47" t="str">
         <v>MTX#46 THEO_PHONG NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P47" t="str">
+        <v/>
+      </c>
+      <c r="Q47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -4606,6 +4852,12 @@
       <c r="O48" t="str">
         <v>MTX#47 THEO_PHONG NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -4653,6 +4905,12 @@
       <c r="O49" t="str">
         <v>MTX#48 THEO_PHONG NT cơ bản — RENO. NT khai thác = TB mua mới đợt 2 (BASIC). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P49" t="str">
+        <v/>
+      </c>
+      <c r="Q49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -4700,6 +4958,12 @@
       <c r="O50" t="str">
         <v>MTX#49 THEO_PHONG không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -4747,10 +5011,16 @@
       <c r="O51" t="str">
         <v>MTX#50 THEO_PHONG không NT — RENO. NT khai thác = TB mua mới đợt 2 (NONE). Đồ chủ bàn giao (nếu có) chỉ ghi nhận, không tính NT.</v>
       </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4758,15 +5028,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G59"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>